<commit_message>
fixed cellFormat add text rotation
</commit_message>
<xml_diff>
--- a/тест/Лист Microsoft Excel.xlsx
+++ b/тест/Лист Microsoft Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\тестовые проекты\ConsoleApp1\тест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A2F5C3-54AE-4FDC-80D9-9FFDDA68E000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D52103-1DF4-4CF7-9C2E-AD807BCB2F30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,21 +26,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="26"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -66,7 +57,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -347,14 +340,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A2:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A1" s="1"/>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>